<commit_message>
Completar calendario a 3+ contenidos por semana y agregar carrusel del 6 nov
- Carrusel del 6 de nov (wifi publico) disenado y subido.
- 3 carruseles nuevos agregados al calendario para llenar semanas con
  menos de 3 contenidos (21 nov, 5 dic, 19 dic) con copys listos;
  carpetas creadas a la espera del diseno.
- Excel y documento de copys actualizados (8 carruseles en total).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/calendario/Calendario_InnovaSites.xlsx
+++ b/calendario/Calendario_InnovaSites.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\santi\AppData\Local\Temp\claude\C--Users-santi\23ce8f98-2a4f-41b9-9b1b-b005d119043d\scratchpad\innovasites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8FB2EFE4-FDD5-4DD0-9118-0F1EC3CC7C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EDF8B75-AF94-4E3F-92CE-12A4A7564FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F3898612-E734-4D40-A571-F70ECF691700}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8EB4941F-ADEE-4878-8728-31620F5A6EB2}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendario" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="120">
   <si>
     <t>#</t>
   </si>
@@ -153,6 +153,24 @@
     <t>Pausa y encuentra las 3 señales</t>
   </si>
   <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>06-nov.-2026</t>
+  </si>
+  <si>
+    <t>Viernes</t>
+  </si>
+  <si>
+    <t>Wifi público: 4 reglas antes de conectarte</t>
+  </si>
+  <si>
+    <t>¿Te conectarías al wifi gratis del centro comercial? Cuéntanos (checklist de 4 reglas, conecta con el reel del wifi del café)</t>
+  </si>
+  <si>
+    <t>#seguridaddigital #wifi #ciberseguridad #tips #innovasites</t>
+  </si>
+  <si>
     <t>09-nov.-2026</t>
   </si>
   <si>
@@ -171,7 +189,7 @@
     <t>¿Real o falso? Vota antes de la respuesta</t>
   </si>
   <si>
-    <t>P2</t>
+    <t>P3</t>
   </si>
   <si>
     <t>14-nov.-2026</t>
@@ -204,6 +222,18 @@
     <t>Elige tu respuesta: A, B o C</t>
   </si>
   <si>
+    <t>P4</t>
+  </si>
+  <si>
+    <t>21-nov.-2026</t>
+  </si>
+  <si>
+    <t>5 frases que usan los estafadores para generar pánico</t>
+  </si>
+  <si>
+    <t>¿Cuál de estas frases ya te dijeron? Cuéntanos sin miedo (conecta con el reel de la llamada del banco)</t>
+  </si>
+  <si>
     <t>23-nov.-2026</t>
   </si>
   <si>
@@ -225,15 +255,12 @@
     <t>#seguridaddigital #estafas #ciberseguridad #tips #innovasites #blackfriday</t>
   </si>
   <si>
-    <t>P3</t>
+    <t>P5</t>
   </si>
   <si>
     <t>27-nov.-2026</t>
   </si>
   <si>
-    <t>Viernes</t>
-  </si>
-  <si>
     <t>Checklist: compra segura en Black Friday</t>
   </si>
   <si>
@@ -261,6 +288,21 @@
     <t>Reto: actívala y comenta LISTO</t>
   </si>
   <si>
+    <t>P6</t>
+  </si>
+  <si>
+    <t>05-dic.-2026</t>
+  </si>
+  <si>
+    <t>Antes y después: así transformamos una web</t>
+  </si>
+  <si>
+    <t>CTA: escríbenos si tu web necesita un cambio (portafolio, llena la semana post-Black Friday)</t>
+  </si>
+  <si>
+    <t>#diseñoweb #portafolio #innovasites #cali #antesydespues</t>
+  </si>
+  <si>
     <t>07-dic.-2026</t>
   </si>
   <si>
@@ -276,7 +318,7 @@
     <t>El trabajo desde casa "fácil"</t>
   </si>
   <si>
-    <t>P4</t>
+    <t>P7</t>
   </si>
   <si>
     <t>12-dic.-2026</t>
@@ -312,6 +354,21 @@
     <t>¿Cuál es la oficial? Vota 1, 2 o 3</t>
   </si>
   <si>
+    <t>P8</t>
+  </si>
+  <si>
+    <t>19-dic.-2026</t>
+  </si>
+  <si>
+    <t>Regalos digitales seguros: lo que debes saber antes de comprar</t>
+  </si>
+  <si>
+    <t>¿Ya compraste una tarjeta de regalo este año? Cuéntanos (conecta con el reel de la tarjeta de regalo navideña)</t>
+  </si>
+  <si>
+    <t>#seguridaddigital #navidad #ciberseguridad #tips #innovasites</t>
+  </si>
+  <si>
     <t>21-dic.-2026</t>
   </si>
   <si>
@@ -333,7 +390,7 @@
     <t>Rojo claro</t>
   </si>
   <si>
-    <t>Posts/carruseles intermedios nuevos (4 en total), intercalados por fecha entre los reels</t>
+    <t>Posts/carruseles intermedios (8 en total), intercalados por fecha para que cada semana tenga al menos 3 contenidos</t>
   </si>
   <si>
     <t>Video listo / Idea / En guion / En edicion / Publicado - actualizar a medida que avance</t>
@@ -342,7 +399,7 @@
     <t>Nota</t>
   </si>
   <si>
-    <t>Los copys completos de los 4 carruseles estan en el documento aparte Copys_Carruseles_InnovaSites.txt</t>
+    <t>Los copys completos de los carruseles estan en el documento aparte Copys_Carruseles_InnovaSites.txt</t>
   </si>
 </sst>
 </file>
@@ -812,8 +869,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F97B1EA7-BE0E-49EB-808B-D2853F252591}">
-  <dimension ref="A1:J22"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC7E947-FA8C-4099-BB84-79D4B8D55E62}">
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
@@ -1020,47 +1077,47 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="s">
+    <row r="7" spans="1:10" ht="140.25" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="5" t="s">
+      <c r="B7" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="C7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>18</v>
+      <c r="D7" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>12</v>
@@ -1072,10 +1129,10 @@
         <v>14</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>17</v>
@@ -1084,79 +1141,79 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="8" t="s">
+    <row r="9" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D10" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
-        <v>6</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>18</v>
+      <c r="G10" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>12</v>
@@ -1168,10 +1225,10 @@
         <v>14</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>17</v>
@@ -1182,13 +1239,13 @@
     </row>
     <row r="12" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>12</v>
@@ -1200,10 +1257,10 @@
         <v>14</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>17</v>
@@ -1212,79 +1269,79 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
-        <v>9</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="5" t="s">
+    <row r="13" spans="1:10" ht="140.25" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>8</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="140.25" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="H14" s="8" t="s">
+      <c r="G14" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="I14" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="J14" s="8" t="s">
+      <c r="H14" s="5" t="s">
         <v>66</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>12</v>
@@ -1305,47 +1362,47 @@
         <v>17</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
-        <v>11</v>
-      </c>
-      <c r="B16" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G16" s="5" t="s">
+    </row>
+    <row r="16" spans="1:10" ht="140.25" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="B16" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="I16" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="C16" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>11</v>
@@ -1360,24 +1417,24 @@
         <v>14</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>20</v>
@@ -1392,10 +1449,10 @@
         <v>14</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>36</v>
+        <v>81</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>17</v>
@@ -1404,12 +1461,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>25</v>
@@ -1424,24 +1481,24 @@
         <v>28</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>17</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>11</v>
@@ -1456,24 +1513,24 @@
         <v>14</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>17</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>20</v>
@@ -1488,10 +1545,10 @@
         <v>14</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>89</v>
+        <v>36</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>17</v>
@@ -1500,35 +1557,163 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3">
+    <row r="22" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
+        <v>14</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>15</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="140.25" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
         <v>16</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C22" s="5" t="s">
+      <c r="B26" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F26" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G22" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="I22" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J22" s="5" t="s">
+      <c r="G26" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J26" s="5" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1538,7 +1723,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97981292-6D2C-46B0-A35B-1B1D16A274AD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D26E6F7C-16F5-4CA7-81D0-1EC3172749D9}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1548,23 +1733,23 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="86.25" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="129" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="186" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1576,7 +1761,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1585,10 +1770,10 @@
     </row>
     <row r="8" spans="1:2" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>